<commit_message>
Residual updates after 24/25, part 2
Various minor updates
</commit_message>
<xml_diff>
--- a/Chap/Database/Presentations/Design/TableTemplate.xlsx
+++ b/Chap/Database/Presentations/Design/TableTemplate.xlsx
@@ -3,12 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11608492-33A5-4582-8389-0D752FB350B7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81A663B-0505-46DF-BA17-434F3F2AE6D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Person" sheetId="1" r:id="rId1"/>
+    <sheet name="Weapon" sheetId="2" r:id="rId2"/>
+    <sheet name="Character" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -20,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="42">
   <si>
     <t>Table name:</t>
   </si>
@@ -83,6 +85,69 @@
   </si>
   <si>
     <t>IsMarried</t>
+  </si>
+  <si>
+    <t>Weapon</t>
+  </si>
+  <si>
+    <t>Weapon description</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Character</t>
+  </si>
+  <si>
+    <t>Character description</t>
+  </si>
+  <si>
+    <t>Race</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Rarity</t>
+  </si>
+  <si>
+    <t>Constraints</t>
+  </si>
+  <si>
+    <t>ItemLevel</t>
+  </si>
+  <si>
+    <t>MinDamage</t>
+  </si>
+  <si>
+    <t>MaxDamage</t>
+  </si>
+  <si>
+    <t>NoOfJewelSockets</t>
+  </si>
+  <si>
+    <t>IsOneHanded</t>
+  </si>
+  <si>
+    <t>double</t>
+  </si>
+  <si>
+    <t>HealthPoints</t>
+  </si>
+  <si>
+    <t>WeaponLeft</t>
+  </si>
+  <si>
+    <t>WeaponRight</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>&lt; MaxDamage</t>
+  </si>
+  <si>
+    <t>&gt; MinDamage</t>
   </si>
 </sst>
 </file>
@@ -601,4 +666,246 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BCCF16F-34B4-42B0-95D4-EF219B778009}">
+  <dimension ref="B3:I15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="8" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="45.77734375" customWidth="1"/>
+    <col min="10" max="10" width="20.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8328A840-D1C3-406A-A2EB-9F99B44B574A}">
+  <dimension ref="B3:I13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="8" width="20.6640625" customWidth="1"/>
+    <col min="9" max="9" width="40.33203125" customWidth="1"/>
+    <col min="10" max="10" width="20.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>